<commit_message>
fix(spark): June L2 sUSDS chi reads at true EoD — supply-side +6,357.21
Same poisoned-cache root cause as #156, one layer deeper: spark's June
EoM pin was always correct (25433938), but the cross-chain chi /
daily-EoD reads valuing the L2 sUSDS POL proxies went through the
poisoned June-30 EoD cache entry (21:10 UTC instead of 23:59:59) on the
machine that generated the committed report — e.g. S37 Base EoM value
+$2,410 on $211M ≈ exactly 2.8h of SSR. Regenerated with the entry
purged; verified in the same full-fleet run that reproduced obex on
HyperSync (debt/balance/position_balance) and keel/skybase/grove
byte-identically.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/spark/2026-06/spark_settlement_june_2026.xlsx
+++ b/settlements/spark/2026-06/spark_settlement_june_2026.xlsx
@@ -491,7 +491,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>11273284.346913</v>
+        <v>11279641.55178227</v>
       </c>
     </row>
     <row r="5">
@@ -517,7 +517,7 @@
     <row r="7">
       <c r="A7" t="inlineStr"/>
       <c r="B7" s="4" t="n">
-        <v>13038911.74687562</v>
+        <v>13045268.95174489</v>
       </c>
     </row>
     <row r="9">
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>8938388.098683022</v>
+        <v>8938388.0890132</v>
       </c>
     </row>
     <row r="11">
@@ -555,7 +555,7 @@
     <row r="12">
       <c r="A12" t="inlineStr"/>
       <c r="B12" s="4" t="n">
-        <v>8959429.599513656</v>
+        <v>8959429.589843834</v>
       </c>
     </row>
     <row r="14">
@@ -577,7 +577,7 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>8938388.098683022</v>
+        <v>8938388.0890132</v>
       </c>
     </row>
     <row r="16">
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>-2736145.682979046</v>
+        <v>-2736145.692648868</v>
       </c>
     </row>
     <row r="17">
@@ -603,7 +603,7 @@
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>171082.354798371</v>
+        <v>171082.3644681933</v>
       </c>
     </row>
     <row r="21">
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B22" s="3" t="n">
-        <v>11273284.346913</v>
+        <v>11279641.55178227</v>
       </c>
     </row>
     <row r="23">
@@ -635,13 +635,13 @@
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>-8938388.098683022</v>
+        <v>-8938388.0890132</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
       <c r="B24" s="4" t="n">
-        <v>1353408.608681825</v>
+        <v>1359765.813551093</v>
       </c>
     </row>
     <row r="26">
@@ -676,7 +676,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-13T18:39:52+00:00</t>
+          <t>2026-07-20T09:02:29+00:00</t>
         </is>
       </c>
     </row>
@@ -873,13 +873,13 @@
         <v>1</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>3016814.373765289</v>
+        <v>3016814.344352271</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>3016814.373765289</v>
+        <v>3016814.344352271</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>9859.197497782963</v>
+        <v>9859.226910800955</v>
       </c>
       <c r="Q2" s="6" t="n">
         <v>0</v>
@@ -938,13 +938,13 @@
         <v>1</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>1346107.850553063</v>
+        <v>1346107.837428922</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>1346107.850553063</v>
+        <v>1346107.837428922</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>-1346107.850553063</v>
+        <v>-1346107.837428922</v>
       </c>
       <c r="Q3" s="6" t="n">
         <v>0</v>
@@ -1003,13 +1003,13 @@
         <v>1</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>1123596.58022099</v>
+        <v>1123596.569266267</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>1123596.58022099</v>
+        <v>1123596.569266267</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>-25108.41107498985</v>
+        <v>-25108.40012026665</v>
       </c>
       <c r="Q4" s="6" t="n">
         <v>0</v>
@@ -1068,13 +1068,13 @@
         <v>1</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>884593.7243238305</v>
+        <v>884593.715699312</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>884593.7243238305</v>
+        <v>884593.715699312</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>111852.6955153982</v>
+        <v>111852.7041399166</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>156917846.5942976</v>
@@ -1137,13 +1137,13 @@
         <v>1</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>579178.9393192878</v>
+        <v>579178.9336724702</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>579178.9393192878</v>
+        <v>579178.9336724702</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>985466.0606807162</v>
+        <v>985466.0663275338</v>
       </c>
       <c r="Q6" s="6" t="n">
         <v>0</v>
@@ -1202,13 +1202,13 @@
         <v>1</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>400430.4143107537</v>
+        <v>400430.4104066796</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>400430.4143107537</v>
+        <v>400430.4104066796</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>113372.8896749099</v>
+        <v>113372.8935789841</v>
       </c>
       <c r="Q7" s="6" t="n">
         <v>89993374.27336854</v>
@@ -1247,19 +1247,19 @@
         <v>143764611.5800855</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>144181483.7745804</v>
+        <v>144183127.2756985</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>416872.1944949473</v>
+        <v>418515.6956130954</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>416872.1944949473</v>
+        <v>418515.6956130954</v>
       </c>
       <c r="I8" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>416872.1944949473</v>
+        <v>418515.6956130954</v>
       </c>
       <c r="K8" s="6" t="n">
         <v>0</v>
@@ -1271,13 +1271,13 @@
         <v>1</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>325101.0995223077</v>
+        <v>325101.0963526713</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>289705.2130477073</v>
+        <v>289705.209878071</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>91771.09497263965</v>
+        <v>93414.59926042407</v>
       </c>
       <c r="Q8" s="6" t="n">
         <v>0</v>
@@ -1312,19 +1312,19 @@
         <v>102351428.4607548</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>201093205.1965842</v>
+        <v>201095497.4250933</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>98741776.73582943</v>
+        <v>98744068.96433853</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>391011.3769401348</v>
+        <v>393303.6054492357</v>
       </c>
       <c r="I9" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>391011.3769401348</v>
+        <v>393303.6054492357</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>0</v>
@@ -1336,13 +1336,13 @@
         <v>1</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>313001.7791243019</v>
+        <v>313001.7760726303</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>278923.2249252826</v>
+        <v>278923.221873611</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>78009.59781583288</v>
+        <v>80301.82937660547</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>0</v>
@@ -1377,19 +1377,19 @@
         <v>76003428.29531698</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>211443541.1594051</v>
+        <v>211445951.3696985</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>135440112.8640881</v>
+        <v>135442523.0743815</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>349807.7689973119</v>
+        <v>352217.9792907777</v>
       </c>
       <c r="I10" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>349807.7689973119</v>
+        <v>352217.9792907777</v>
       </c>
       <c r="K10" s="6" t="n">
         <v>0</v>
@@ -1401,13 +1401,13 @@
         <v>1</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>283882.836955894</v>
+        <v>283882.8341881231</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>252974.6527518328</v>
+        <v>252974.6499840619</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>65924.93204141795</v>
+        <v>68335.14510265466</v>
       </c>
       <c r="Q10" s="6" t="n">
         <v>0</v>
@@ -1466,13 +1466,13 @@
         <v>1</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>237652.8049211904</v>
+        <v>237652.8026041482</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>237652.8049211904</v>
+        <v>237652.8026041482</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>177441.378266123</v>
+        <v>177441.3805831652</v>
       </c>
       <c r="Q11" s="6" t="n">
         <v>0</v>
@@ -1531,13 +1531,13 @@
         <v>1</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>226133.71963043</v>
+        <v>226133.7174256953</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>226133.71963043</v>
+        <v>226133.7174256953</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>-199366.3806834299</v>
+        <v>-199366.3784786953</v>
       </c>
       <c r="Q12" s="6" t="n">
         <v>0</v>
@@ -1596,13 +1596,13 @@
         <v>1</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>218592.6048086293</v>
+        <v>218592.6026774182</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>218592.6048086293</v>
+        <v>218592.6026774182</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>-188466.4602882971</v>
+        <v>-188466.458157086</v>
       </c>
       <c r="Q13" s="6" t="n">
         <v>0</v>
@@ -1722,13 +1722,13 @@
         <v>1</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>44521.89678920271</v>
+        <v>44521.89635512782</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>44521.89678920271</v>
+        <v>44521.89635512782</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>51125.42290101229</v>
+        <v>51125.42333508717</v>
       </c>
       <c r="Q15" s="6" t="n">
         <v>0</v>
@@ -1787,13 +1787,13 @@
         <v>1</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>27137.96448612331</v>
+        <v>27137.96422153645</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>27137.96448612331</v>
+        <v>27137.96422153645</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>10216.38188987669</v>
+        <v>10216.38215446355</v>
       </c>
       <c r="Q16" s="6" t="n">
         <v>0</v>
@@ -1852,13 +1852,13 @@
         <v>1</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>25275.145187121</v>
+        <v>25275.14494069606</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>25275.145187121</v>
+        <v>25275.14494069606</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>18870.94278013413</v>
+        <v>18870.94302655907</v>
       </c>
       <c r="Q17" s="6" t="n">
         <v>0</v>
@@ -1986,13 +1986,13 @@
         <v>1</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>10973.53816437875</v>
+        <v>10973.53805739011</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>10973.53816437875</v>
+        <v>10973.53805739011</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>-10973.53816437875</v>
+        <v>-10973.53805739011</v>
       </c>
       <c r="Q19" s="6" t="n">
         <v>0</v>
@@ -2051,13 +2051,13 @@
         <v>1</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>10924.52731975241</v>
+        <v>10924.52721324161</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>10924.52731975241</v>
+        <v>10924.52721324161</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>-10924.52731975241</v>
+        <v>-10924.52721324161</v>
       </c>
       <c r="Q20" s="6" t="n">
         <v>0</v>
@@ -2116,13 +2116,13 @@
         <v>1</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>10914.12814718641</v>
+        <v>10914.128040777</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>10914.12814718641</v>
+        <v>10914.128040777</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-10914.12814718641</v>
+        <v>-10914.128040777</v>
       </c>
       <c r="Q21" s="6" t="n">
         <v>0</v>
@@ -2181,13 +2181,13 @@
         <v>1</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>10876.08734013992</v>
+        <v>10876.08723410139</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>10876.08734013992</v>
+        <v>10876.08723410139</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>-10876.08734013992</v>
+        <v>-10876.08723410139</v>
       </c>
       <c r="Q22" s="6" t="n">
         <v>0</v>
@@ -2222,43 +2222,43 @@
         <v>985396.9281006901</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>104354426.4993414</v>
+        <v>104355616.018357</v>
       </c>
       <c r="G23" s="6" t="n">
-        <v>103369029.5712408</v>
+        <v>103370219.0902563</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>2857.341423254798</v>
+        <v>2868.606371807529</v>
       </c>
       <c r="I23" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J23" s="6" t="n">
-        <v>2857.341423254798</v>
+        <v>2868.606371807529</v>
       </c>
       <c r="K23" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>4430936.00242794</v>
+        <v>4430975.277563506</v>
       </c>
       <c r="M23" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>10019.86615809035</v>
+        <v>10019.95487495214</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>8928.937688320224</v>
+        <v>8929.016735359764</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>-7162.52473483555</v>
+        <v>-7151.348503144608</v>
       </c>
       <c r="Q23" s="6" t="n">
         <v>0</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>1090.928469770123</v>
+        <v>1090.938139592373</v>
       </c>
       <c r="S23" t="inlineStr"/>
     </row>
@@ -2311,13 +2311,13 @@
         <v>1</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>3301.209848374132</v>
+        <v>3301.209816188345</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>3301.209848374132</v>
+        <v>3301.209816188345</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>1609.906493111088</v>
+        <v>1609.906525296875</v>
       </c>
       <c r="Q24" s="6" t="n">
         <v>0</v>
@@ -2445,13 +2445,13 @@
         <v>1</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>437.1879686660595</v>
+        <v>437.1879644036105</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>437.1879686660595</v>
+        <v>437.1879644036105</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>253.1499077627124</v>
+        <v>253.1499120251614</v>
       </c>
       <c r="Q26" s="6" t="n">
         <v>0</v>
@@ -2579,13 +2579,13 @@
         <v>1</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>1.220837798409625</v>
+        <v>1.22083778650683</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>1.220837798409625</v>
+        <v>1.22083778650683</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>96.39293744541818</v>
+        <v>96.39293745732098</v>
       </c>
       <c r="Q28" s="6" t="n">
         <v>0</v>
@@ -2644,13 +2644,13 @@
         <v>1</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>0.6419890593344861</v>
+        <v>0.6419890530752891</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>0.6419890593344861</v>
+        <v>0.6419890530752891</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>-0.6419890593344861</v>
+        <v>-0.6419890530752891</v>
       </c>
       <c r="Q29" s="6" t="n">
         <v>0</v>
@@ -2709,13 +2709,13 @@
         <v>1</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>0.2257115602198127</v>
+        <v>0.225711558019194</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>0.2257115602198127</v>
+        <v>0.225711558019194</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>0.08505712848573202</v>
+        <v>0.08505713068635073</v>
       </c>
       <c r="Q30" s="6" t="n">
         <v>0</v>
@@ -2774,13 +2774,13 @@
         <v>1</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>0.04953910018384292</v>
+        <v>0.04953909970085183</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>0.04953910018384292</v>
+        <v>0.04953909970085183</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>-0.04935510355092702</v>
+        <v>-0.04935510306793594</v>
       </c>
       <c r="Q31" s="6" t="n">
         <v>0</v>
@@ -2839,13 +2839,13 @@
         <v>1</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>0.0226496070682828</v>
+        <v>0.02264960684745605</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>0.0226496070682828</v>
+        <v>0.02264960684745605</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>-8.685264607068282</v>
+        <v>-8.685264606847456</v>
       </c>
       <c r="Q32" s="6" t="n">
         <v>0</v>
@@ -2904,13 +2904,13 @@
         <v>1</v>
       </c>
       <c r="N33" s="6" t="n">
-        <v>0.01337190464628485</v>
+        <v>0.01337190451591287</v>
       </c>
       <c r="O33" s="6" t="n">
-        <v>0.01337190464628485</v>
+        <v>0.01337190451591287</v>
       </c>
       <c r="P33" s="6" t="n">
-        <v>-0.001804904646284854</v>
+        <v>-0.001804904515912871</v>
       </c>
       <c r="Q33" s="6" t="n">
         <v>0</v>
@@ -2969,13 +2969,13 @@
         <v>1</v>
       </c>
       <c r="N34" s="6" t="n">
-        <v>0.0003508812881901634</v>
+        <v>0.0003508812847691781</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>0.0003508812881901634</v>
+        <v>0.0003508812847691781</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>9.111871180983658e-05</v>
+        <v>9.111871523082189e-05</v>
       </c>
       <c r="Q34" s="6" t="n">
         <v>0</v>
@@ -3034,13 +3034,13 @@
         <v>1</v>
       </c>
       <c r="N35" s="6" t="n">
-        <v>0.0001310877929629464</v>
+        <v>0.0001310877916848805</v>
       </c>
       <c r="O35" s="6" t="n">
-        <v>0.0001310877929629464</v>
+        <v>0.0001310877916848805</v>
       </c>
       <c r="P35" s="6" t="n">
-        <v>2.791220703705357e-05</v>
+        <v>2.791220831511948e-05</v>
       </c>
       <c r="Q35" s="6" t="n">
         <v>0</v>
@@ -3099,13 +3099,13 @@
         <v>1</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>1.43889255744144e-05</v>
+        <v>1.438892543412677e-05</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>1.43889255744144e-05</v>
+        <v>1.438892543412677e-05</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>-2.388925574414396e-06</v>
+        <v>-2.388925434126771e-06</v>
       </c>
       <c r="Q36" s="6" t="n">
         <v>0</v>
@@ -3164,13 +3164,13 @@
         <v>1</v>
       </c>
       <c r="N37" s="6" t="n">
-        <v>1.299464233742441e-05</v>
+        <v>1.299464221073062e-05</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>1.299464233742441e-05</v>
+        <v>1.299464221073062e-05</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>-1.180289297087241e-05</v>
+        <v>-1.180289284417862e-05</v>
       </c>
       <c r="Q37" s="6" t="n">
         <v>0</v>
@@ -3229,13 +3229,13 @@
         <v>1</v>
       </c>
       <c r="N38" s="6" t="n">
-        <v>3.855589832528139e-06</v>
+        <v>3.855589794937317e-06</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>3.855589832528139e-06</v>
+        <v>3.855589794937317e-06</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>1.444101674718614e-07</v>
+        <v>1.444102050626837e-07</v>
       </c>
       <c r="Q38" s="6" t="n">
         <v>0</v>
@@ -3294,13 +3294,13 @@
         <v>1</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>2.804392482394191e-06</v>
+        <v>2.804392455052222e-06</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>2.804392482394191e-06</v>
+        <v>2.804392455052222e-06</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>-2.804392482394191e-06</v>
+        <v>-2.804392455052222e-06</v>
       </c>
       <c r="Q39" s="6" t="n">
         <v>0</v>
@@ -3359,13 +3359,13 @@
         <v>1</v>
       </c>
       <c r="N40" s="6" t="n">
-        <v>1.179682205733403e-06</v>
+        <v>1.179682194231862e-06</v>
       </c>
       <c r="O40" s="6" t="n">
-        <v>1.179682205733403e-06</v>
+        <v>1.179682194231862e-06</v>
       </c>
       <c r="P40" s="6" t="n">
-        <v>-7.131520660224029e-07</v>
+        <v>-7.13152054520862e-07</v>
       </c>
       <c r="Q40" s="6" t="n">
         <v>0</v>
@@ -3424,13 +3424,13 @@
         <v>1</v>
       </c>
       <c r="N41" s="6" t="n">
-        <v>1.693661699975317e-07</v>
+        <v>1.693661683462633e-07</v>
       </c>
       <c r="O41" s="6" t="n">
-        <v>1.693661699975317e-07</v>
+        <v>1.693661683462633e-07</v>
       </c>
       <c r="P41" s="6" t="n">
-        <v>-1.693661699975317e-07</v>
+        <v>-1.693661683462633e-07</v>
       </c>
       <c r="Q41" s="6" t="n">
         <v>0</v>
@@ -4826,7 +4826,7 @@
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>8938388.098683022</v>
+        <v>8938388.0890132</v>
       </c>
     </row>
     <row r="25">
@@ -4846,7 +4846,7 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>8959429.599513656</v>
+        <v>8959429.589843834</v>
       </c>
     </row>
     <row r="28">
@@ -4873,7 +4873,7 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>8938388.098683022</v>
+        <v>8938388.0890132</v>
       </c>
     </row>
     <row r="32">
@@ -4883,7 +4883,7 @@
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>-2736145.682979046</v>
+        <v>-2736145.692648868</v>
       </c>
     </row>
     <row r="33" ht="60" customHeight="1">
@@ -4900,7 +4900,7 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>171082.354798371</v>
+        <v>171082.3644681933</v>
       </c>
     </row>
     <row r="37">

</xml_diff>